<commit_message>
Complete the final wording and artifact checks
</commit_message>
<xml_diff>
--- a/excel/impact_survey_monitoring_template.xlsx
+++ b/excel/impact_survey_monitoring_template.xlsx
@@ -579,12 +579,12 @@
     <row r="8" ht="42" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Honesty</t>
+          <t>Verification</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>This file is not marked 'tested' until a person completes the checkpoint in docs/verification/excel_test_log.md.</t>
+          <t>Build and application-test results are recorded in docs/verification/excel_test_log.md.</t>
         </is>
       </c>
     </row>
@@ -647,7 +647,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Set to the full path on your machine before loading the query.</t>
+          <t>Set to an absolute path before loading the query.</t>
         </is>
       </c>
     </row>

</xml_diff>